<commit_message>
refactor: use inequality in summarize_bootstrap_replicas()
</commit_message>
<xml_diff>
--- a/data/final/bootstrap_summary_control.xlsx
+++ b/data/final/bootstrap_summary_control.xlsx
@@ -492,19 +492,19 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>2899519.0593944</v>
+        <v>2898085.6253058</v>
       </c>
       <c r="E2" t="n">
-        <v>2899888.6565</v>
+        <v>2897332.681</v>
       </c>
       <c r="F2" t="n">
-        <v>2720185.08825</v>
+        <v>2720240.4348</v>
       </c>
       <c r="G2" t="n">
-        <v>3084258.076475</v>
+        <v>3081412.644475</v>
       </c>
       <c r="H2" t="n">
-        <v>92611.461620794</v>
+        <v>91796.94693387992</v>
       </c>
       <c r="I2" t="n">
         <v>10000</v>
@@ -527,19 +527,19 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2897414.183102934</v>
+        <v>2895000.698604569</v>
       </c>
       <c r="E3" t="n">
-        <v>2888926.784537881</v>
+        <v>2885416.251114222</v>
       </c>
       <c r="F3" t="n">
-        <v>2576797.116200646</v>
+        <v>2569131.725341174</v>
       </c>
       <c r="G3" t="n">
-        <v>3256175.08538124</v>
+        <v>3266902.545003101</v>
       </c>
       <c r="H3" t="n">
-        <v>175154.0760958772</v>
+        <v>175686.1770983407</v>
       </c>
       <c r="I3" t="n">
         <v>10000</v>
@@ -562,19 +562,19 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>8425684830924.003</v>
+        <v>8411891591181.093</v>
       </c>
       <c r="E4" t="n">
-        <v>8345897966918.255</v>
+        <v>8325626942234.666</v>
       </c>
       <c r="F4" t="n">
-        <v>6639883378643.938</v>
+        <v>6600437822296.741</v>
       </c>
       <c r="G4" t="n">
-        <v>10602676186688.89</v>
+        <v>10672652238752.44</v>
       </c>
       <c r="H4" t="n">
-        <v>1024012222621.899</v>
+        <v>1025895051886.287</v>
       </c>
       <c r="I4" t="n">
         <v>10000</v>
@@ -597,19 +597,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>38.2042369</v>
+        <v>38.2080608</v>
       </c>
       <c r="E5" t="n">
-        <v>38.2</v>
+        <v>38.20950000000001</v>
       </c>
       <c r="F5" t="n">
-        <v>37.592975</v>
+        <v>37.585</v>
       </c>
       <c r="G5" t="n">
-        <v>38.835</v>
+        <v>38.834</v>
       </c>
       <c r="H5" t="n">
-        <v>0.3150079703444471</v>
+        <v>0.3169435773548387</v>
       </c>
       <c r="I5" t="n">
         <v>10000</v>
@@ -632,19 +632,19 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>10.01594772173391</v>
+        <v>10.01955647892116</v>
       </c>
       <c r="E6" t="n">
-        <v>10.01479501117245</v>
+        <v>10.02088699547729</v>
       </c>
       <c r="F6" t="n">
-        <v>9.505897226198666</v>
+        <v>9.510098721701999</v>
       </c>
       <c r="G6" t="n">
-        <v>10.53781381000861</v>
+        <v>10.53111430445221</v>
       </c>
       <c r="H6" t="n">
-        <v>0.262095576438801</v>
+        <v>0.261825507435799</v>
       </c>
       <c r="I6" t="n">
         <v>10000</v>
@@ -667,19 +667,19 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100.3878959862863</v>
+        <v>100.4600577753754</v>
       </c>
       <c r="E7" t="n">
-        <v>100.2961191191191</v>
+        <v>100.4181761761762</v>
       </c>
       <c r="F7" t="n">
-        <v>90.36208208208208</v>
+        <v>90.44197770270269</v>
       </c>
       <c r="G7" t="n">
-        <v>111.0455198948949</v>
+        <v>110.9043684934935</v>
       </c>
       <c r="H7" t="n">
-        <v>5.254531347938346</v>
+        <v>5.249605331010418</v>
       </c>
       <c r="I7" t="n">
         <v>10000</v>
@@ -702,19 +702,19 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.491813391666667</v>
+        <v>2.492966296666667</v>
       </c>
       <c r="E8" t="n">
-        <v>2.488208333333333</v>
+        <v>2.488183333333333</v>
       </c>
       <c r="F8" t="n">
-        <v>2.325682916666667</v>
+        <v>2.322933333333333</v>
       </c>
       <c r="G8" t="n">
-        <v>2.680704166666667</v>
+        <v>2.690385</v>
       </c>
       <c r="H8" t="n">
-        <v>0.09092717290985952</v>
+        <v>0.09341498496835558</v>
       </c>
       <c r="I8" t="n">
         <v>10000</v>
@@ -737,19 +737,19 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2.871110419171816</v>
+        <v>2.879746124523172</v>
       </c>
       <c r="E9" t="n">
-        <v>2.866262297220524</v>
+        <v>2.873555218745019</v>
       </c>
       <c r="F9" t="n">
-        <v>1.955473015187357</v>
+        <v>1.975028119964702</v>
       </c>
       <c r="G9" t="n">
-        <v>3.801865574784849</v>
+        <v>3.847314070868554</v>
       </c>
       <c r="H9" t="n">
-        <v>0.471544317267899</v>
+        <v>0.4820223492670366</v>
       </c>
       <c r="I9" t="n">
         <v>10000</v>
@@ -772,19 +772,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>8.465606846820293</v>
+        <v>8.52526005234462</v>
       </c>
       <c r="E10" t="n">
-        <v>8.215459556779001</v>
+        <v>8.257319601545989</v>
       </c>
       <c r="F10" t="n">
-        <v>3.82387471443666</v>
+        <v>3.900736074657991</v>
       </c>
       <c r="G10" t="n">
-        <v>14.45418186111111</v>
+        <v>14.80182556012262</v>
       </c>
       <c r="H10" t="n">
-        <v>2.738933859614809</v>
+        <v>2.818626088632025</v>
       </c>
       <c r="I10" t="n">
         <v>10000</v>
@@ -807,7 +807,7 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>0.5879497</v>
+        <v>0.5880529999999999</v>
       </c>
       <c r="E11" t="n">
         <v>0.588</v>
@@ -816,10 +816,10 @@
         <v>0.5570000000000001</v>
       </c>
       <c r="G11" t="n">
-        <v>0.618</v>
+        <v>0.619</v>
       </c>
       <c r="H11" t="n">
-        <v>0.01562896658034808</v>
+        <v>0.01555842528856137</v>
       </c>
       <c r="I11" t="n">
         <v>10000</v>
@@ -842,19 +842,19 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>0.4100612</v>
+        <v>0.4099403</v>
       </c>
       <c r="E12" t="n">
         <v>0.41</v>
       </c>
       <c r="F12" t="n">
-        <v>0.38</v>
+        <v>0.379</v>
       </c>
       <c r="G12" t="n">
-        <v>0.441</v>
+        <v>0.4410249999999996</v>
       </c>
       <c r="H12" t="n">
-        <v>0.01563585311232664</v>
+        <v>0.01553847741376334</v>
       </c>
       <c r="I12" t="n">
         <v>10000</v>
@@ -877,7 +877,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.002311831706183202</v>
+        <v>0.002315334025614432</v>
       </c>
       <c r="E13" t="n">
         <v>0.002000000000000002</v>
@@ -889,7 +889,7 @@
         <v>0.005000000000000115</v>
       </c>
       <c r="H13" t="n">
-        <v>0.001247774051179905</v>
+        <v>0.00125821519706031</v>
       </c>
       <c r="I13" t="n">
         <v>10000</v>
@@ -912,19 +912,19 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>0.4940175999999999</v>
+        <v>0.4942098</v>
       </c>
       <c r="E14" t="n">
         <v>0.494</v>
       </c>
       <c r="F14" t="n">
-        <v>0.463</v>
+        <v>0.464</v>
       </c>
       <c r="G14" t="n">
         <v>0.525</v>
       </c>
       <c r="H14" t="n">
-        <v>0.01589674686519509</v>
+        <v>0.01568437387715532</v>
       </c>
       <c r="I14" t="n">
         <v>10000</v>
@@ -947,7 +947,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0.5059824000000001</v>
+        <v>0.5057902000000001</v>
       </c>
       <c r="E15" t="n">
         <v>0.506</v>
@@ -956,10 +956,10 @@
         <v>0.475</v>
       </c>
       <c r="G15" t="n">
-        <v>0.5369999999999999</v>
+        <v>0.536</v>
       </c>
       <c r="H15" t="n">
-        <v>0.01589674686519509</v>
+        <v>0.01568437387715532</v>
       </c>
       <c r="I15" t="n">
         <v>10000</v>
@@ -982,7 +982,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.6669251</v>
+        <v>0.6668282999999999</v>
       </c>
       <c r="E16" t="n">
         <v>0.667</v>
@@ -994,7 +994,7 @@
         <v>0.696</v>
       </c>
       <c r="H16" t="n">
-        <v>0.01479209148792214</v>
+        <v>0.01488551567691548</v>
       </c>
       <c r="I16" t="n">
         <v>10000</v>
@@ -1017,7 +1017,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.3330749</v>
+        <v>0.3331717</v>
       </c>
       <c r="E17" t="n">
         <v>0.333</v>
@@ -1029,7 +1029,7 @@
         <v>0.362</v>
       </c>
       <c r="H17" t="n">
-        <v>0.01479209148792214</v>
+        <v>0.01488551567691548</v>
       </c>
       <c r="I17" t="n">
         <v>10000</v>
@@ -1052,7 +1052,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.1519922</v>
+        <v>0.1520853</v>
       </c>
       <c r="E18" t="n">
         <v>0.152</v>
@@ -1064,7 +1064,7 @@
         <v>0.175</v>
       </c>
       <c r="H18" t="n">
-        <v>0.01150047674040192</v>
+        <v>0.01128910839290822</v>
       </c>
       <c r="I18" t="n">
         <v>10000</v>
@@ -1087,7 +1087,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.3586557634964539</v>
+        <v>0.3587590433205887</v>
       </c>
       <c r="E19" t="n">
         <v>0.35902089075707</v>
@@ -1099,7 +1099,7 @@
         <v>0.3799671038392666</v>
       </c>
       <c r="H19" t="n">
-        <v>0.01115254001071532</v>
+        <v>0.01094948057253978</v>
       </c>
       <c r="I19" t="n">
         <v>10000</v>
@@ -1122,7 +1122,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.1287583234</v>
+        <v>0.1288279303</v>
       </c>
       <c r="E20" t="n">
         <v>0.128896</v>
@@ -1134,7 +1134,7 @@
         <v>0.144375</v>
       </c>
       <c r="H20" t="n">
-        <v>0.00799196889813138</v>
+        <v>0.007845975925368625</v>
       </c>
       <c r="I20" t="n">
         <v>10000</v>
@@ -1157,7 +1157,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.5541133</v>
+        <v>0.5543777</v>
       </c>
       <c r="E21" t="n">
         <v>0.554</v>
@@ -1169,7 +1169,7 @@
         <v>0.585</v>
       </c>
       <c r="H21" t="n">
-        <v>0.0156832349818508</v>
+        <v>0.0159356279177732</v>
       </c>
       <c r="I21" t="n">
         <v>10000</v>
@@ -1192,7 +1192,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.4968126277665002</v>
+        <v>0.4967755727364511</v>
       </c>
       <c r="E22" t="n">
         <v>0.4970754469896899</v>
@@ -1204,7 +1204,7 @@
         <v>0.4994707198625361</v>
       </c>
       <c r="H22" t="n">
-        <v>0.001739164803665324</v>
+        <v>0.001782568407120686</v>
       </c>
       <c r="I22" t="n">
         <v>10000</v>
@@ -1227,7 +1227,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.2468258115</v>
+        <v>0.2467891469</v>
       </c>
       <c r="E23" t="n">
         <v>0.247084</v>
@@ -1239,7 +1239,7 @@
         <v>0.249471</v>
       </c>
       <c r="H23" t="n">
-        <v>0.001725550131550338</v>
+        <v>0.001768391147468631</v>
       </c>
       <c r="I23" t="n">
         <v>10000</v>

</xml_diff>